<commit_message>
Rerunning k sweep, now that chunk size and chunk overlap have been solidified
</commit_message>
<xml_diff>
--- a/1. RAG/RAG_evaluation.xlsx
+++ b/1. RAG/RAG_evaluation.xlsx
@@ -645,7 +645,7 @@
         <v>0.8</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>0.7064</v>
+        <v>0.6657</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>8</v>
@@ -726,10 +726,10 @@
         <v>2</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>0.5742</v>
+        <v>0.5793</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>8</v>
@@ -758,7 +758,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>The barriers to HIV &amp; AIDS treatment in Bosnia and Herzegovina include the availability of antiretroviral medication that belongs to an older generation of products, and the funding through mandatory health insurance, which implies that treatment is considered aesthetic rather than vital. Additionally, there is a societal stigma, as it is viewed as unacceptable to have a relative who is LGBTI.</t>
+          <t>The barriers to HIV &amp; AIDS treatment in Bosnia and Herzegovina include the availability of antiretroviral medication from an older generation of products and the perception that certain medical procedures related to treatment are aesthetic rather than vital, which affects funding through mandatory health insurance. Additionally, societal attitudes deeming it unacceptable to have a relative who is LGBTI may contribute to stigma and discrimination in accessing treatment.</t>
         </is>
       </c>
       <c r="D7" s="4" t="n">
@@ -774,19 +774,19 @@
         <v>0.5783</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="I7" s="4" t="b">
         <v>1</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>0.66</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="K7" s="4" t="n">
         <v>0.8179999999999999</v>
       </c>
       <c r="L7" s="4" t="n">
-        <v>14.2</v>
+        <v>-4.8</v>
       </c>
     </row>
     <row r="8">
@@ -813,7 +813,7 @@
         <v>0.8</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>0.5152</v>
+        <v>0.51</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>8</v>
@@ -855,7 +855,7 @@
         <v>0.8</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.3549</v>
+        <v>0.3295</v>
       </c>
       <c r="H9" s="4" t="n">
         <v>8</v>
@@ -1198,7 +1198,7 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Question b1_c — In your opinion, how widespread are expressions of hatred and aversion towards lesbian, gay, bisexual and/or transgender in public in the country where you live? | Poland responses (Transgender): Very widespread: 42%, Fairly widespread: 44%, Fairly rare: 12%, Very rare: 1%, Don`t know: 1%</t>
+          <t>Question c1a_d — In your opinion, in the country where you live, how widespread is discrimination because a person is Transgender? | Poland responses (Bisexual men): Very widespread: 69%, Fairly widespread: 16%, Fairly rare: 5%, Very rare: 1%, Don`t know: 9%</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>C:\Users\RAZER\Desktop\portfolio-projects\1. RAG\data\3_txt_KB\LGBT_EU\by_country\LGBT_Survey_DailyLife\b1_c_answer_by_Poland.txt</t>
+          <t>C:\Users\RAZER\Desktop\portfolio-projects\1. RAG\data\3_txt_KB\LGBT_EU\by_country\LGBT_Survey_DailyLife\c1a_d_answer_by_Poland.txt</t>
         </is>
       </c>
       <c r="E13" s="4" t="b">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Question b1_c — In your opinion, how widespread are expressions of hatred and aversion towards lesbian, gay, bisexual and/or transgender in public in the country where you live? | Poland responses (Transgender): Very widespread: 42%, Fairly widespread: 44%, Fairly rare: 12%, Very rare: 1%, Don`t know: 1%</t>
+          <t>Question c1a_d — In your opinion, in the country where you live, how widespread is discrimination because a person is Transgender? | Poland responses (Bisexual men): Very widespread: 69%, Fairly widespread: 16%, Fairly rare: 5%, Very rare: 1%, Don`t know: 9%</t>
         </is>
       </c>
     </row>
@@ -1240,13 +1240,17 @@
       <c r="C14" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="D14" s="3" t="inlineStr"/>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>C:\Users\RAZER\Desktop\portfolio-projects\1. RAG\data\3_txt_KB\LGBT_EU\by_country\LGBT_Survey_DailyLife\c1a_d_answer_by_Poland.txt</t>
+        </is>
+      </c>
       <c r="E14" s="2" t="b">
         <v>1</v>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Question b1_c — In your opinion, how widespread are expressions of hatred and aversion towards lesbian, gay, bisexual and/or transgender in public in the country where you live? | Poland responses (Transgender): Very widespread: 42%, Fairly widespread: 44%, Fairly rare: 12%, Very rare: 1%, Don`t know: 1%</t>
+          <t>Question c1a_d — In your opinion, in the country where you live, how widespread is discrimination because a person is Transgender? | Poland responses (Bisexual men): Very widespread: 69%, Fairly widespread: 16%, Fairly rare: 5%, Very rare: 1%, Don`t know: 9%</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1268,7 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>C:\Users\RAZER\Desktop\portfolio-projects\1. RAG\data\3_txt_KB\LGBT_EU\by_country\LGBT_Survey_DailyLife\b1_c_answer_by_Poland.txt</t>
+          <t>C:\Users\RAZER\Desktop\portfolio-projects\1. RAG\data\3_txt_KB\LGBT_EU\by_country\LGBT_Survey_DailyLife\c1a_d_answer_by_Poland.txt</t>
         </is>
       </c>
       <c r="E15" s="4" t="b">
@@ -1272,7 +1276,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Question b1_c — In your opinion, how widespread are expressions of hatred and aversion towards lesbian, gay, bisexual and/or transgender in public in the country where you live? | Poland responses (Transgender): Very widespread: 42%, Fairly widespread: 44%, Fairly rare: 12%, Very rare: 1%, Don`t know: 1%</t>
+          <t>Question c1a_d — In your opinion, in the country where you live, how widespread is discrimination because a person is Transgender? | Poland responses (Bisexual men): Very widespread: 69%, Fairly widespread: 16%, Fairly rare: 5%, Very rare: 1%, Don`t know: 9%</t>
         </is>
       </c>
     </row>
@@ -1290,7 +1294,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>C:\Users\RAZER\Desktop\portfolio-projects\1. RAG\data\3_txt_KB\LGBT_EU\by_country\LGBT_Survey_DailyLife\b1_c_answer_by_Poland.txt</t>
+          <t>C:\Users\RAZER\Desktop\portfolio-projects\1. RAG\data\3_txt_KB\LGBT_EU\by_country\LGBT_Survey_DailyLife\c1a_d_answer_by_Poland.txt</t>
         </is>
       </c>
       <c r="E16" s="2" t="b">
@@ -1298,7 +1302,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Question b1_c — In your opinion, how widespread are expressions of hatred and aversion towards lesbian, gay, bisexual and/or transgender in public in the country where you live? | Poland responses (Transgender): Very widespread: 42%, Fairly widespread: 44%, Fairly rare: 12%, Very rare: 1%, Don`t know: 1%</t>
+          <t>Question c1a_d — In your opinion, in the country where you live, how widespread is discrimination because a person is Transgender? | Poland responses (Bisexual men): Very widespread: 69%, Fairly widespread: 16%, Fairly rare: 5%, Very rare: 1%, Don`t know: 9%</t>
         </is>
       </c>
     </row>
@@ -1432,11 +1436,43 @@
       <c r="C22" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D22" s="3" t="inlineStr"/>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>C:\Users\RAZER\Desktop\portfolio-projects\1. RAG\data\3_txt_KB\UNICEF_Immunization\HEPB3_Belgium.txt</t>
+        </is>
+      </c>
       <c r="E22" s="2" t="b">
         <v>0</v>
       </c>
       <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>HEPB3 coverage in Belgium (2017): 97.0%
+HEPB3 coverage in Belgium (2018): 97.0%
+HEPB3 coverage in Belgium (2019): 97.0%
+HEPB3 coverage in Belgium (2020): 97.0%
+HEPB3 coverage in Belgium (2021): 97.0%
+HEPB3 coverage in Belgium (2022): 97.0%
+HEPB3 coverage in Belgium (2023): 97.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>What is the HIV prevalence rate among adults in Belgium?</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" s="5" t="inlineStr"/>
+      <c r="E23" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
         <is>
           <t>HEPB3 coverage in Belgium (2011): 97.0%
 HEPB3 coverage in Belgium (2012): 98.0%
@@ -1453,27 +1489,27 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="4" t="n">
+    <row r="24">
+      <c r="A24" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>What is the HIV prevalence rate among adults in Belgium?</t>
         </is>
       </c>
-      <c r="C23" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="C24" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>C:\Users\RAZER\Desktop\portfolio-projects\1. RAG\data\3_txt_KB\UNICEF_Immunization\HEPB3_Belgium.txt</t>
         </is>
       </c>
-      <c r="E23" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="E24" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
         <is>
           <t>HEPB3 coverage in Belgium (2011): 97.0%
 HEPB3 coverage in Belgium (2012): 98.0%
@@ -1490,27 +1526,27 @@
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="2" t="n">
+    <row r="25">
+      <c r="A25" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>What is the HIV prevalence rate among adults in Belgium?</t>
         </is>
       </c>
-      <c r="C24" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="C25" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>C:\Users\RAZER\Desktop\portfolio-projects\1. RAG\data\3_txt_KB\UNICEF_Immunization\HEPB3_Belgium.txt</t>
         </is>
       </c>
-      <c r="E24" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
+      <c r="E25" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
         <is>
           <t>HEPB3 coverage in Belgium (2011): 97.0%
 HEPB3 coverage in Belgium (2012): 98.0%
@@ -1527,27 +1563,27 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="4" t="n">
+    <row r="26">
+      <c r="A26" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>What is the HIV prevalence rate among adults in Belgium?</t>
         </is>
       </c>
-      <c r="C25" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="C26" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>C:\Users\RAZER\Desktop\portfolio-projects\1. RAG\data\3_txt_KB\UNICEF_Immunization\HEPB3_Belgium.txt</t>
         </is>
       </c>
-      <c r="E25" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="E26" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
         <is>
           <t>HEPB3 coverage in Belgium (2011): 97.0%
 HEPB3 coverage in Belgium (2012): 98.0%
@@ -1564,43 +1600,6 @@
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>What is the HIV prevalence rate among adults in Belgium?</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>C:\Users\RAZER\Desktop\portfolio-projects\1. RAG\data\3_txt_KB\UNICEF_Immunization\HEPB3_Belgium.txt</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>HEPB3 coverage in Belgium (2011): 97.0%
-HEPB3 coverage in Belgium (2012): 98.0%
-HEPB3 coverage in Belgium (2013): 98.0%
-HEPB3 coverage in Belgium (2014): 98.0%
-HEPB3 coverage in Belgium (2015): 98.0%
-HEPB3 coverage in Belgium (2016): 97.0%
-HEPB3 coverage in Belgium (2017): 97.0%
-HEPB3 coverage in Belgium (2018): 97.0%
-HEPB3 coverage in Belgium (2019): 97.0%
-HEPB3 coverage in Belgium (2020): 97.0%
-HEPB3 coverage in Belgium (2021): 97.0%
-HEPB3 coverage in Belgium (2022): 97.0%</t>
-        </is>
-      </c>
-    </row>
     <row r="27">
       <c r="A27" s="4" t="n">
         <v>6</v>
@@ -1788,25 +1787,28 @@
       <c r="C32" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D32" s="3" t="inlineStr"/>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>C:\Users\RAZER\Desktop\portfolio-projects\1. RAG\data\3_txt_KB\UNICEF_Immunization\MCV2_Slovenia.txt</t>
+        </is>
+      </c>
       <c r="E32" s="2" t="b">
         <v>0</v>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>MCV1 coverage in Malta (2000): 74.0%
-MCV1 coverage in Malta (2001): 70.0%
-MCV1 coverage in Malta (2002): 65.0%
-MCV1 coverage in Malta (2003): 90.0%
-MCV1 coverage in Malta (2004): 94.0%
-MCV1 coverage in Malta (2005): 86.0%
-MCV1 coverage in Malta (2006): 94.0%
-MCV1 coverage in Malta (2007): 79.0%
-MCV1 coverage in Malta (2008): 78.0%
-MCV1 coverage in Malta (2009): 82.0%
-MCV1 coverage in Malta (2010): 73.0%
-MCV1 coverage in Malta (2011): 84.0%
-MCV1 coverage in Malta (2012): 93.0%</t>
+          <t>MCV2 coverage in Slovenia (2000): 98.0%
+MCV2 coverage in Slovenia (2001): 98.0%
+MCV2 coverage in Slovenia (2002): 98.0%
+MCV2 coverage in Slovenia (2003): 98.0%
+MCV2 coverage in Slovenia (2004): 99.0%
+MCV2 coverage in Slovenia (2005): 99.0%
+MCV2 coverage in Slovenia (2006): 99.0%
+MCV2 coverage in Slovenia (2007): 98.0%
+MCV2 coverage in Slovenia (2008): 98.0%
+MCV2 coverage in Slovenia (2009): 98.0%
+MCV2 coverage in Slovenia (2010): 96.0%
+MCV2 coverage in Slovenia (2011): 96.0%</t>
         </is>
       </c>
     </row>
@@ -1822,25 +1824,28 @@
       <c r="C33" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="D33" s="5" t="inlineStr"/>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>C:\Users\RAZER\Desktop\portfolio-projects\1. RAG\data\3_txt_KB\UNICEF_Immunization\MCV2_Slovenia.txt</t>
+        </is>
+      </c>
       <c r="E33" s="4" t="b">
         <v>1</v>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>MCV1 coverage in Malta (2000): 74.0%
-MCV1 coverage in Malta (2001): 70.0%
-MCV1 coverage in Malta (2002): 65.0%
-MCV1 coverage in Malta (2003): 90.0%
-MCV1 coverage in Malta (2004): 94.0%
-MCV1 coverage in Malta (2005): 86.0%
-MCV1 coverage in Malta (2006): 94.0%
-MCV1 coverage in Malta (2007): 79.0%
-MCV1 coverage in Malta (2008): 78.0%
-MCV1 coverage in Malta (2009): 82.0%
-MCV1 coverage in Malta (2010): 73.0%
-MCV1 coverage in Malta (2011): 84.0%
-MCV1 coverage in Malta (2012): 93.0%</t>
+          <t>MCV2 coverage in Slovenia (2000): 98.0%
+MCV2 coverage in Slovenia (2001): 98.0%
+MCV2 coverage in Slovenia (2002): 98.0%
+MCV2 coverage in Slovenia (2003): 98.0%
+MCV2 coverage in Slovenia (2004): 99.0%
+MCV2 coverage in Slovenia (2005): 99.0%
+MCV2 coverage in Slovenia (2006): 99.0%
+MCV2 coverage in Slovenia (2007): 98.0%
+MCV2 coverage in Slovenia (2008): 98.0%
+MCV2 coverage in Slovenia (2009): 98.0%
+MCV2 coverage in Slovenia (2010): 96.0%
+MCV2 coverage in Slovenia (2011): 96.0%</t>
         </is>
       </c>
     </row>
@@ -1856,29 +1861,24 @@
       <c r="C34" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>C:\Users\RAZER\Desktop\portfolio-projects\1. RAG\data\3_txt_KB\UNICEF_Immunization\MCV1_Malta.txt</t>
-        </is>
-      </c>
+      <c r="D34" s="3" t="inlineStr"/>
       <c r="E34" s="2" t="b">
         <v>1</v>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>MCV1 coverage in Malta (2000): 74.0%
-MCV1 coverage in Malta (2001): 70.0%
-MCV1 coverage in Malta (2002): 65.0%
-MCV1 coverage in Malta (2003): 90.0%
-MCV1 coverage in Malta (2004): 94.0%
-MCV1 coverage in Malta (2005): 86.0%
-MCV1 coverage in Malta (2006): 94.0%
-MCV1 coverage in Malta (2007): 79.0%
-MCV1 coverage in Malta (2008): 78.0%
-MCV1 coverage in Malta (2009): 82.0%
-MCV1 coverage in Malta (2010): 73.0%
-MCV1 coverage in Malta (2011): 84.0%
-MCV1 coverage in Malta (2012): 93.0%</t>
+          <t>MCV2 coverage in Slovenia (2000): 98.0%
+MCV2 coverage in Slovenia (2001): 98.0%
+MCV2 coverage in Slovenia (2002): 98.0%
+MCV2 coverage in Slovenia (2003): 98.0%
+MCV2 coverage in Slovenia (2004): 99.0%
+MCV2 coverage in Slovenia (2005): 99.0%
+MCV2 coverage in Slovenia (2006): 99.0%
+MCV2 coverage in Slovenia (2007): 98.0%
+MCV2 coverage in Slovenia (2008): 98.0%
+MCV2 coverage in Slovenia (2009): 98.0%
+MCV2 coverage in Slovenia (2010): 96.0%
+MCV2 coverage in Slovenia (2011): 96.0%</t>
         </is>
       </c>
     </row>
@@ -1894,29 +1894,24 @@
       <c r="C35" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>C:\Users\RAZER\Desktop\portfolio-projects\1. RAG\data\3_txt_KB\UNICEF_Immunization\MCV1_Malta.txt</t>
-        </is>
-      </c>
+      <c r="D35" s="5" t="inlineStr"/>
       <c r="E35" s="4" t="b">
         <v>1</v>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>MCV1 coverage in Malta (2000): 74.0%
-MCV1 coverage in Malta (2001): 70.0%
-MCV1 coverage in Malta (2002): 65.0%
-MCV1 coverage in Malta (2003): 90.0%
-MCV1 coverage in Malta (2004): 94.0%
-MCV1 coverage in Malta (2005): 86.0%
-MCV1 coverage in Malta (2006): 94.0%
-MCV1 coverage in Malta (2007): 79.0%
-MCV1 coverage in Malta (2008): 78.0%
-MCV1 coverage in Malta (2009): 82.0%
-MCV1 coverage in Malta (2010): 73.0%
-MCV1 coverage in Malta (2011): 84.0%
-MCV1 coverage in Malta (2012): 93.0%</t>
+          <t>MCV2 coverage in Slovenia (2000): 98.0%
+MCV2 coverage in Slovenia (2001): 98.0%
+MCV2 coverage in Slovenia (2002): 98.0%
+MCV2 coverage in Slovenia (2003): 98.0%
+MCV2 coverage in Slovenia (2004): 99.0%
+MCV2 coverage in Slovenia (2005): 99.0%
+MCV2 coverage in Slovenia (2006): 99.0%
+MCV2 coverage in Slovenia (2007): 98.0%
+MCV2 coverage in Slovenia (2008): 98.0%
+MCV2 coverage in Slovenia (2009): 98.0%
+MCV2 coverage in Slovenia (2010): 96.0%
+MCV2 coverage in Slovenia (2011): 96.0%</t>
         </is>
       </c>
     </row>
@@ -1934,7 +1929,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>C:\Users\RAZER\Desktop\portfolio-projects\1. RAG\data\3_txt_KB\UNICEF_Immunization\MCV1_Malta.txt</t>
+          <t>C:\Users\RAZER\Desktop\portfolio-projects\1. RAG\data\3_txt_KB\UNICEF_Immunization\MCV2_Slovenia.txt</t>
         </is>
       </c>
       <c r="E36" s="2" t="b">
@@ -1942,19 +1937,18 @@
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>MCV1 coverage in Malta (2000): 74.0%
-MCV1 coverage in Malta (2001): 70.0%
-MCV1 coverage in Malta (2002): 65.0%
-MCV1 coverage in Malta (2003): 90.0%
-MCV1 coverage in Malta (2004): 94.0%
-MCV1 coverage in Malta (2005): 86.0%
-MCV1 coverage in Malta (2006): 94.0%
-MCV1 coverage in Malta (2007): 79.0%
-MCV1 coverage in Malta (2008): 78.0%
-MCV1 coverage in Malta (2009): 82.0%
-MCV1 coverage in Malta (2010): 73.0%
-MCV1 coverage in Malta (2011): 84.0%
-MCV1 coverage in Malta (2012): 93.0%</t>
+          <t>MCV2 coverage in Slovenia (2000): 98.0%
+MCV2 coverage in Slovenia (2001): 98.0%
+MCV2 coverage in Slovenia (2002): 98.0%
+MCV2 coverage in Slovenia (2003): 98.0%
+MCV2 coverage in Slovenia (2004): 99.0%
+MCV2 coverage in Slovenia (2005): 99.0%
+MCV2 coverage in Slovenia (2006): 99.0%
+MCV2 coverage in Slovenia (2007): 98.0%
+MCV2 coverage in Slovenia (2008): 98.0%
+MCV2 coverage in Slovenia (2009): 98.0%
+MCV2 coverage in Slovenia (2010): 96.0%
+MCV2 coverage in Slovenia (2011): 96.0%</t>
         </is>
       </c>
     </row>
@@ -1976,8 +1970,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>Question d3_d — Do you know of any organisation in the country where you live that can offer support or advice to people who have been discriminated against because they are Transgender? | Transgender responses in Portugal: Yes: 89%, No: 11%
-Question d3_d — Do you know of any organisation in the country where you live that can offer support or advice to people who have been discriminated against because they are Transgender? | Transgender responses in Romania: Yes: 75%, No: 25%</t>
+          <t>Question b1_i — In your opinion, how widespread are positive measures to promote respect for the human rights of transgender people in the country where you live? * | Denmark responses (Transgender): Very widespread: 1%, Fairly widespread: 11%, Fairly rare: 27%, Very rare: 52%, Don`t know: 9%</t>
         </is>
       </c>
     </row>
@@ -1995,7 +1988,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>C:\Users\RAZER\Desktop\portfolio-projects\1. RAG\data\3_txt_KB\LGBT_EU\by_subset\LGBT_Survey_RightsAwareness\d3_d_answer_by_Transgender.txt</t>
+          <t>C:\Users\RAZER\Desktop\portfolio-projects\1. RAG\data\3_txt_KB\LGBT_EU\by_country\LGBT_Survey_DailyLife\b1_i_answer_by_Denmark.txt</t>
         </is>
       </c>
       <c r="E38" s="2" t="b">
@@ -2003,8 +1996,7 @@
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>Question d3_d — Do you know of any organisation in the country where you live that can offer support or advice to people who have been discriminated against because they are Transgender? | Transgender responses in Portugal: Yes: 89%, No: 11%
-Question d3_d — Do you know of any organisation in the country where you live that can offer support or advice to people who have been discriminated against because they are Transgender? | Transgender responses in Romania: Yes: 75%, No: 25%</t>
+          <t>Question b1_i — In your opinion, how widespread are positive measures to promote respect for the human rights of transgender people in the country where you live? * | Denmark responses (Transgender): Very widespread: 1%, Fairly widespread: 11%, Fairly rare: 27%, Very rare: 52%, Don`t know: 9%</t>
         </is>
       </c>
     </row>
@@ -2022,7 +2014,7 @@
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>C:\Users\RAZER\Desktop\portfolio-projects\1. RAG\data\3_txt_KB\LGBT_EU\by_subset\LGBT_Survey_RightsAwareness\d3_d_answer_by_Transgender.txt</t>
+          <t>C:\Users\RAZER\Desktop\portfolio-projects\1. RAG\data\3_txt_KB\LGBT_EU\by_country\LGBT_Survey_DailyLife\b1_i_answer_by_Denmark.txt</t>
         </is>
       </c>
       <c r="E39" s="4" t="b">
@@ -2030,8 +2022,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>Question d3_d — Do you know of any organisation in the country where you live that can offer support or advice to people who have been discriminated against because they are Transgender? | Transgender responses in Portugal: Yes: 89%, No: 11%
-Question d3_d — Do you know of any organisation in the country where you live that can offer support or advice to people who have been discriminated against because they are Transgender? | Transgender responses in Romania: Yes: 75%, No: 25%</t>
+          <t>Question b1_i — In your opinion, how widespread are positive measures to promote respect for the human rights of transgender people in the country where you live? * | Denmark responses (Transgender): Very widespread: 1%, Fairly widespread: 11%, Fairly rare: 27%, Very rare: 52%, Don`t know: 9%</t>
         </is>
       </c>
     </row>
@@ -2049,7 +2040,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>C:\Users\RAZER\Desktop\portfolio-projects\1. RAG\data\3_txt_KB\LGBT_EU\by_subset\LGBT_Survey_RightsAwareness\d3_d_answer_by_Transgender.txt</t>
+          <t>C:\Users\RAZER\Desktop\portfolio-projects\1. RAG\data\3_txt_KB\LGBT_EU\by_country\LGBT_Survey_DailyLife\b1_i_answer_by_Denmark.txt</t>
         </is>
       </c>
       <c r="E40" s="2" t="b">
@@ -2057,8 +2048,7 @@
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>Question d3_d — Do you know of any organisation in the country where you live that can offer support or advice to people who have been discriminated against because they are Transgender? | Transgender responses in Portugal: Yes: 89%, No: 11%
-Question d3_d — Do you know of any organisation in the country where you live that can offer support or advice to people who have been discriminated against because they are Transgender? | Transgender responses in Romania: Yes: 75%, No: 25%</t>
+          <t>Question b1_i — In your opinion, how widespread are positive measures to promote respect for the human rights of transgender people in the country where you live? * | Denmark responses (Transgender): Very widespread: 1%, Fairly widespread: 11%, Fairly rare: 27%, Very rare: 52%, Don`t know: 9%</t>
         </is>
       </c>
     </row>
@@ -2076,7 +2066,7 @@
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>C:\Users\RAZER\Desktop\portfolio-projects\1. RAG\data\3_txt_KB\LGBT_EU\by_subset\LGBT_Survey_RightsAwareness\d3_d_answer_by_Transgender.txt</t>
+          <t>C:\Users\RAZER\Desktop\portfolio-projects\1. RAG\data\3_txt_KB\LGBT_EU\by_country\LGBT_Survey_DailyLife\b1_i_answer_by_Denmark.txt</t>
         </is>
       </c>
       <c r="E41" s="4" t="b">
@@ -2084,8 +2074,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>Question d3_d — Do you know of any organisation in the country where you live that can offer support or advice to people who have been discriminated against because they are Transgender? | Transgender responses in Portugal: Yes: 89%, No: 11%
-Question d3_d — Do you know of any organisation in the country where you live that can offer support or advice to people who have been discriminated against because they are Transgender? | Transgender responses in Romania: Yes: 75%, No: 25%</t>
+          <t>Question b1_i — In your opinion, how widespread are positive measures to promote respect for the human rights of transgender people in the country where you live? * | Denmark responses (Transgender): Very widespread: 1%, Fairly widespread: 11%, Fairly rare: 27%, Very rare: 52%, Don`t know: 9%</t>
         </is>
       </c>
     </row>

</xml_diff>